<commit_message>
models refactoring and timeseries fix
</commit_message>
<xml_diff>
--- a/output/tables/model_results.xlsx
+++ b/output/tables/model_results.xlsx
@@ -14,30 +14,23 @@
     <sheet name="Case_FE_Clash" sheetId="5" r:id="rId5"/>
     <sheet name="Case_FE_Clash_Interaction" sheetId="6" r:id="rId6"/>
     <sheet name="TWFE" sheetId="7" r:id="rId7"/>
-    <sheet name="TWFE_Clashes" sheetId="8" r:id="rId8"/>
-    <sheet name="TWFE_Clashes_Interaction" sheetId="9" r:id="rId9"/>
-    <sheet name="TWFE_By_Case" sheetId="10" r:id="rId10"/>
-    <sheet name="TWFE_By_Case_Interaction" sheetId="11" r:id="rId11"/>
-    <sheet name="Political_Violence_FE" sheetId="12" r:id="rId12"/>
-    <sheet name="Civilian_Targeting_FE" sheetId="13" r:id="rId13"/>
-    <sheet name="Homicides_FE" sheetId="14" r:id="rId14"/>
-    <sheet name="Terrorism_FE" sheetId="15" r:id="rId15"/>
-    <sheet name="Extortion_FE" sheetId="16" r:id="rId16"/>
-    <sheet name="Political_Violence_OLS" sheetId="17" r:id="rId17"/>
-    <sheet name="Civilian_Targeting_OLS" sheetId="18" r:id="rId18"/>
-    <sheet name="Homicides_OLS" sheetId="19" r:id="rId19"/>
-    <sheet name="Terrorism_OLS" sheetId="20" r:id="rId20"/>
-    <sheet name="Extortion_OLS" sheetId="21" r:id="rId21"/>
-    <sheet name="Political_Violence_TWFE" sheetId="22" r:id="rId22"/>
-    <sheet name="Civilian_Targeting_TWFE" sheetId="23" r:id="rId23"/>
-    <sheet name="Homicides_TWFE" sheetId="24" r:id="rId24"/>
-    <sheet name="Terrorism_TWFE" sheetId="25" r:id="rId25"/>
-    <sheet name="Extortion_TWFE" sheetId="26" r:id="rId26"/>
-    <sheet name="Political_Violence_TWFE_Inter" sheetId="27" r:id="rId27"/>
-    <sheet name="Civilian_Targeting_TWFE_Inter" sheetId="28" r:id="rId28"/>
-    <sheet name="Homicides_TWFE_Interaction" sheetId="29" r:id="rId29"/>
-    <sheet name="Terrorism_TWFE_Interaction" sheetId="30" r:id="rId30"/>
-    <sheet name="Extortion_TWFE_Interaction" sheetId="31" r:id="rId31"/>
+    <sheet name="TWFE_Clash" sheetId="8" r:id="rId8"/>
+    <sheet name="TWFE_Clash_Interaction" sheetId="9" r:id="rId9"/>
+    <sheet name="Political_Violence_OLS" sheetId="10" r:id="rId10"/>
+    <sheet name="Civilian_Targeting_OLS" sheetId="11" r:id="rId11"/>
+    <sheet name="Homicide_OLS" sheetId="12" r:id="rId12"/>
+    <sheet name="Terrorism_OLS" sheetId="13" r:id="rId13"/>
+    <sheet name="Extortion_OLS" sheetId="14" r:id="rId14"/>
+    <sheet name="Political_Violence_FE" sheetId="15" r:id="rId15"/>
+    <sheet name="Civilian_Targeting_FE" sheetId="16" r:id="rId16"/>
+    <sheet name="Homicide_FE" sheetId="17" r:id="rId17"/>
+    <sheet name="Terrorism_FE" sheetId="18" r:id="rId18"/>
+    <sheet name="Extortion_FE" sheetId="19" r:id="rId19"/>
+    <sheet name="Political_Violence_TWFE" sheetId="20" r:id="rId20"/>
+    <sheet name="Civilian_Targeting_TWFE" sheetId="21" r:id="rId21"/>
+    <sheet name="Homicide_TWFE" sheetId="22" r:id="rId22"/>
+    <sheet name="Terrorism_TWFE" sheetId="23" r:id="rId23"/>
+    <sheet name="Extortion_TWFE" sheetId="24" r:id="rId24"/>
   </sheets>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -509,97 +502,97 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>TWFE by Case</t>
+          <t>OLS: Political violence</t>
         </is>
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>tr_buenaventura</t>
+          <t>(Intercept)</t>
         </is>
       </c>
       <c r="C2">
-        <v>1.880814855161695</v>
+        <v>8.348837209302326</v>
       </c>
       <c r="D2">
-        <v>0.8682313245132496</v>
+        <v>0.87093105518905</v>
       </c>
       <c r="E2">
-        <v>2.166260076156689</v>
+        <v>9.586105765272169</v>
       </c>
       <c r="F2">
-        <v>0.03049481200095025</v>
+        <v>4.152540055386222E-19</v>
       </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>TWFE by Case</t>
+          <t>OLS: Political violence</t>
         </is>
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>tr_arauca</t>
+          <t>treatment_dummy</t>
         </is>
       </c>
       <c r="C3">
-        <v>-1.451721753402127</v>
+        <v>-6.31180017226528</v>
       </c>
       <c r="D3">
-        <v>1.06327162743322</v>
+        <v>1.7817268156033</v>
       </c>
       <c r="E3">
-        <v>-1.365334798697339</v>
+        <v>-3.542518480942366</v>
       </c>
       <c r="F3">
-        <v>0.1724130126694128</v>
+        <v>0.000460978817299831</v>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>TWFE by Case</t>
+          <t>OLS: Political violence</t>
         </is>
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>tr_tumaco</t>
+          <t>clash_dummy</t>
         </is>
       </c>
       <c r="C4">
-        <v>0.891491816630591</v>
+        <v>0.8511627906976681</v>
       </c>
       <c r="D4">
-        <v>1.14513259514815</v>
+        <v>1.131540226453705</v>
       </c>
       <c r="E4">
-        <v>0.7785053193034431</v>
+        <v>0.7522161128687826</v>
       </c>
       <c r="F4">
-        <v>0.4364302147579442</v>
+        <v>0.452524961914135</v>
       </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>TWFE by Case</t>
+          <t>OLS: Political violence</t>
         </is>
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>clash_dummy</t>
+          <t>treatment_dummy:clash_dummy</t>
         </is>
       </c>
       <c r="C5">
-        <v>5.208281587926979</v>
+        <v>6.637223901078853</v>
       </c>
       <c r="D5">
-        <v>0.7823179192212029</v>
+        <v>2.191358816977466</v>
       </c>
       <c r="E5">
-        <v>6.657500052039995</v>
+        <v>3.028816572465095</v>
       </c>
       <c r="F5">
-        <v>4.291000974055795E-11</v>
+        <v>0.002673800192365788</v>
       </c>
     </row>
   </sheetData>
@@ -609,7 +602,7 @@
 
 <file path=xl/worksheets/sheet11.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:F6"/>
+  <dimension ref="A1:F5"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <sheetData>
     <row r="1" s="1" customFormat="1">
@@ -647,121 +640,97 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>TWFE by Case + clash + interaction</t>
+          <t>OLS: Civilian targeting</t>
         </is>
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>tr_buenaventura</t>
+          <t>(Intercept)</t>
         </is>
       </c>
       <c r="C2">
-        <v>3.229104018520571</v>
+        <v>4.046511627906985</v>
       </c>
       <c r="D2">
-        <v>1.071571326809892</v>
+        <v>0.5634861405513617</v>
       </c>
       <c r="E2">
-        <v>3.013428912971882</v>
+        <v>7.181208794146279</v>
       </c>
       <c r="F2">
-        <v>0.002639336845799129</v>
+        <v>5.722438820968966E-12</v>
       </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>TWFE by Case + clash + interaction</t>
+          <t>OLS: Civilian targeting</t>
         </is>
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>tr_arauca</t>
+          <t>treatment_dummy</t>
         </is>
       </c>
       <c r="C3">
-        <v>-1.007894863920107</v>
+        <v>-3.342807924203267</v>
       </c>
       <c r="D3">
-        <v>1.08168989801198</v>
+        <v>1.152764459206522</v>
       </c>
       <c r="E3">
-        <v>-0.9317780130631711</v>
+        <v>-2.899818690198178</v>
       </c>
       <c r="F3">
-        <v>0.3516456462484965</v>
+        <v>0.004016279507387538</v>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>TWFE by Case + clash + interaction</t>
+          <t>OLS: Civilian targeting</t>
         </is>
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>tr_tumaco</t>
+          <t>clash_dummy</t>
         </is>
       </c>
       <c r="C4">
-        <v>0.6098471655663574</v>
+        <v>1.641488372093018</v>
       </c>
       <c r="D4">
-        <v>1.150911814881571</v>
+        <v>0.7320984035235818</v>
       </c>
       <c r="E4">
-        <v>0.5298817491321965</v>
+        <v>2.242169036556495</v>
       </c>
       <c r="F4">
-        <v>0.5962955853481702</v>
+        <v>0.02569848204661665</v>
       </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>TWFE by Case + clash + interaction</t>
+          <t>OLS: Civilian targeting</t>
         </is>
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>clash_dummy</t>
+          <t>treatment_dummy:clash_dummy</t>
         </is>
       </c>
       <c r="C5">
-        <v>5.683145979848571</v>
+        <v>4.349723178440565</v>
       </c>
       <c r="D5">
-        <v>0.8120037087747729</v>
+        <v>1.41779342346886</v>
       </c>
       <c r="E5">
-        <v>6.998916283798547</v>
+        <v>3.067952711896679</v>
       </c>
       <c r="F5">
-        <v>4.359840385622874E-12</v>
-      </c>
-    </row>
-    <row r="6">
-      <c r="A6" t="inlineStr">
-        <is>
-          <t>TWFE by Case + clash + interaction</t>
-        </is>
-      </c>
-      <c r="B6" t="inlineStr">
-        <is>
-          <t>tr_buenaventura:clash_dummy</t>
-        </is>
-      </c>
-      <c r="C6">
-        <v>-3.003158111020457</v>
-      </c>
-      <c r="D6">
-        <v>1.403011533517305</v>
-      </c>
-      <c r="E6">
-        <v>-2.140508498523627</v>
-      </c>
-      <c r="F6">
-        <v>0.03252225865476369</v>
+        <v>0.002356806383161828</v>
       </c>
     </row>
   </sheetData>
@@ -771,7 +740,7 @@
 
 <file path=xl/worksheets/sheet12.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:F3"/>
+  <dimension ref="A1:F5"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <sheetData>
     <row r="1" s="1" customFormat="1">
@@ -809,49 +778,97 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>Case FE + Clash: Political violence</t>
+          <t>OLS: Homicide</t>
         </is>
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>treatment_dummy</t>
+          <t>(Intercept)</t>
         </is>
       </c>
       <c r="C2">
-        <v>-0.9752412941851217</v>
+        <v>8.790697674418611</v>
       </c>
       <c r="D2">
-        <v>0.785376321147221</v>
+        <v>0.7967544101561371</v>
       </c>
       <c r="E2">
-        <v>-1.241750315008937</v>
+        <v>11.03313337505836</v>
       </c>
       <c r="F2">
-        <v>0.2153251817230532</v>
+        <v>1.30935984495446E-23</v>
       </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>Case FE + Clash: Political violence</t>
+          <t>OLS: Homicide</t>
         </is>
       </c>
       <c r="B3" t="inlineStr">
         <is>
+          <t>treatment_dummy</t>
+        </is>
+      </c>
+      <c r="C3">
+        <v>-2.012919896640838</v>
+      </c>
+      <c r="D3">
+        <v>1.629978273902785</v>
+      </c>
+      <c r="E3">
+        <v>-1.234936642327843</v>
+      </c>
+      <c r="F3">
+        <v>0.2179276728555414</v>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" t="inlineStr">
+        <is>
+          <t>OLS: Homicide</t>
+        </is>
+      </c>
+      <c r="B4" t="inlineStr">
+        <is>
           <t>clash_dummy</t>
         </is>
       </c>
-      <c r="C3">
-        <v>3.408350566454843</v>
-      </c>
-      <c r="D3">
-        <v>0.8799981176191883</v>
-      </c>
-      <c r="E3">
-        <v>3.873133928599808</v>
-      </c>
-      <c r="F3">
-        <v>0.0001326595612870174</v>
+      <c r="C4">
+        <v>-0.8776541961577377</v>
+      </c>
+      <c r="D4">
+        <v>1.053352146454991</v>
+      </c>
+      <c r="E4">
+        <v>-0.8332011275729992</v>
+      </c>
+      <c r="F4">
+        <v>0.4054677475967221</v>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="inlineStr">
+        <is>
+          <t>OLS: Homicide</t>
+        </is>
+      </c>
+      <c r="B5" t="inlineStr">
+        <is>
+          <t>treatment_dummy:clash_dummy</t>
+        </is>
+      </c>
+      <c r="C5">
+        <v>4.752050331423441</v>
+      </c>
+      <c r="D5">
+        <v>2.078074881609994</v>
+      </c>
+      <c r="E5">
+        <v>2.286756061332004</v>
+      </c>
+      <c r="F5">
+        <v>0.02298429436082683</v>
       </c>
     </row>
   </sheetData>
@@ -861,7 +878,7 @@
 
 <file path=xl/worksheets/sheet13.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:F3"/>
+  <dimension ref="A1:F5"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <sheetData>
     <row r="1" s="1" customFormat="1">
@@ -899,49 +916,97 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>Case FE + Clash: Civilian targeting</t>
+          <t>OLS: Terrorism</t>
         </is>
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>treatment_dummy</t>
+          <t>(Intercept)</t>
         </is>
       </c>
       <c r="C2">
-        <v>-0.06546320724547638</v>
+        <v>7.470588235294124</v>
       </c>
       <c r="D2">
-        <v>0.5445361870063766</v>
+        <v>0.638526072340958</v>
       </c>
       <c r="E2">
-        <v>-0.1202182863279751</v>
+        <v>11.69973875601591</v>
       </c>
       <c r="F2">
-        <v>0.904392907118065</v>
+        <v>1.32848696982739E-22</v>
       </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>Case FE + Clash: Civilian targeting</t>
+          <t>OLS: Terrorism</t>
         </is>
       </c>
       <c r="B3" t="inlineStr">
         <is>
+          <t>treatment_dummy</t>
+        </is>
+      </c>
+      <c r="C3">
+        <v>-6.327731092436986</v>
+      </c>
+      <c r="D3">
+        <v>1.837991979363508</v>
+      </c>
+      <c r="E3">
+        <v>-3.442741406645453</v>
+      </c>
+      <c r="F3">
+        <v>0.0007555550410819314</v>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" t="inlineStr">
+        <is>
+          <t>OLS: Terrorism</t>
+        </is>
+      </c>
+      <c r="B4" t="inlineStr">
+        <is>
           <t>clash_dummy</t>
         </is>
       </c>
-      <c r="C3">
-        <v>3.683077937862959</v>
-      </c>
-      <c r="D3">
-        <v>0.6101416692079211</v>
-      </c>
-      <c r="E3">
-        <v>6.03643075655575</v>
-      </c>
-      <c r="F3">
-        <v>4.773103735172649E-09</v>
+      <c r="C4">
+        <v>-3.739819004524874</v>
+      </c>
+      <c r="D4">
+        <v>0.8986603399280008</v>
+      </c>
+      <c r="E4">
+        <v>-4.161548961673888</v>
+      </c>
+      <c r="F4">
+        <v>5.432344955858865E-05</v>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="inlineStr">
+        <is>
+          <t>OLS: Terrorism</t>
+        </is>
+      </c>
+      <c r="B5" t="inlineStr">
+        <is>
+          <t>treatment_dummy:clash_dummy</t>
+        </is>
+      </c>
+      <c r="C5">
+        <v>6.407772672478516</v>
+      </c>
+      <c r="D5">
+        <v>2.083284826792342</v>
+      </c>
+      <c r="E5">
+        <v>3.075802497128843</v>
+      </c>
+      <c r="F5">
+        <v>0.002515940551178633</v>
       </c>
     </row>
   </sheetData>
@@ -951,7 +1016,7 @@
 
 <file path=xl/worksheets/sheet14.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:F3"/>
+  <dimension ref="A1:F5"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <sheetData>
     <row r="1" s="1" customFormat="1">
@@ -989,49 +1054,97 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>Case FE + Clash: Homicides</t>
+          <t>OLS: Extortion</t>
         </is>
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>treatment_dummy</t>
+          <t>(Intercept)</t>
         </is>
       </c>
       <c r="C2">
-        <v>-1.31406025339287</v>
+        <v>8.895348837209283</v>
       </c>
       <c r="D2">
-        <v>0.8860979929929363</v>
+        <v>0.6843068515922716</v>
       </c>
       <c r="E2">
-        <v>-1.482973964261474</v>
+        <v>12.99906440584548</v>
       </c>
       <c r="F2">
-        <v>0.1392519463482527</v>
+        <v>1.042582182794389E-29</v>
       </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>Case FE + Clash: Homicides</t>
+          <t>OLS: Extortion</t>
         </is>
       </c>
       <c r="B3" t="inlineStr">
         <is>
+          <t>treatment_dummy</t>
+        </is>
+      </c>
+      <c r="C3">
+        <v>4.69724375538335</v>
+      </c>
+      <c r="D3">
+        <v>1.399936149157487</v>
+      </c>
+      <c r="E3">
+        <v>3.355327139891527</v>
+      </c>
+      <c r="F3">
+        <v>0.0009191333590784011</v>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" t="inlineStr">
+        <is>
+          <t>OLS: Extortion</t>
+        </is>
+      </c>
+      <c r="B4" t="inlineStr">
+        <is>
           <t>clash_dummy</t>
         </is>
       </c>
-      <c r="C3">
-        <v>5.026394569680934</v>
-      </c>
-      <c r="D3">
-        <v>0.9105507525854878</v>
-      </c>
-      <c r="E3">
-        <v>5.520169584626231</v>
-      </c>
-      <c r="F3">
-        <v>7.969835261877551E-08</v>
+      <c r="C4">
+        <v>-1.0792568831863</v>
+      </c>
+      <c r="D4">
+        <v>0.9649711151328827</v>
+      </c>
+      <c r="E4">
+        <v>-1.118434392761777</v>
+      </c>
+      <c r="F4">
+        <v>0.2644814163270539</v>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="inlineStr">
+        <is>
+          <t>OLS: Extortion</t>
+        </is>
+      </c>
+      <c r="B5" t="inlineStr">
+        <is>
+          <t>treatment_dummy:clash_dummy</t>
+        </is>
+      </c>
+      <c r="C5">
+        <v>-6.180002376072965</v>
+      </c>
+      <c r="D5">
+        <v>1.8060201741882</v>
+      </c>
+      <c r="E5">
+        <v>-3.42189000122928</v>
+      </c>
+      <c r="F5">
+        <v>0.0007290341761693907</v>
       </c>
     </row>
   </sheetData>
@@ -1041,7 +1154,7 @@
 
 <file path=xl/worksheets/sheet15.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:F3"/>
+  <dimension ref="A1:F4"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <sheetData>
     <row r="1" s="1" customFormat="1">
@@ -1079,7 +1192,7 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>Case FE + Clash: Terrorism</t>
+          <t>Case FE: Political violence</t>
         </is>
       </c>
       <c r="B2" t="inlineStr">
@@ -1088,22 +1201,22 @@
         </is>
       </c>
       <c r="C2">
-        <v>-1.171870864369913</v>
+        <v>1.247717798282903</v>
       </c>
       <c r="D2">
-        <v>0.9366910725251997</v>
+        <v>1.390402019937213</v>
       </c>
       <c r="E2">
-        <v>-1.251075086272253</v>
+        <v>0.8973791611286975</v>
       </c>
       <c r="F2">
-        <v>0.2129643871842708</v>
+        <v>0.3702584486201337</v>
       </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>Case FE + Clash: Terrorism</t>
+          <t>Case FE: Political violence</t>
         </is>
       </c>
       <c r="B3" t="inlineStr">
@@ -1112,16 +1225,40 @@
         </is>
       </c>
       <c r="C3">
-        <v>-1.304245069584256</v>
+        <v>4.317554710464798</v>
       </c>
       <c r="D3">
-        <v>0.8630446876306543</v>
+        <v>0.994172073358047</v>
       </c>
       <c r="E3">
-        <v>-1.511213832003119</v>
+        <v>4.342864606809217</v>
       </c>
       <c r="F3">
-        <v>0.1329561739593671</v>
+        <v>1.944131802766714E-05</v>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" t="inlineStr">
+        <is>
+          <t>Case FE: Political violence</t>
+        </is>
+      </c>
+      <c r="B4" t="inlineStr">
+        <is>
+          <t>treatment_dummy:clash_dummy</t>
+        </is>
+      </c>
+      <c r="C4">
+        <v>-3.296013594136837</v>
+      </c>
+      <c r="D4">
+        <v>1.704883659401272</v>
+      </c>
+      <c r="E4">
+        <v>-1.933277720131557</v>
+      </c>
+      <c r="F4">
+        <v>0.05417186893631662</v>
       </c>
     </row>
   </sheetData>
@@ -1131,7 +1268,7 @@
 
 <file path=xl/worksheets/sheet16.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:F3"/>
+  <dimension ref="A1:F4"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <sheetData>
     <row r="1" s="1" customFormat="1">
@@ -1169,7 +1306,7 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>Case FE + Clash: Extortion</t>
+          <t>Case FE: Civilian targeting</t>
         </is>
       </c>
       <c r="B2" t="inlineStr">
@@ -1178,22 +1315,22 @@
         </is>
       </c>
       <c r="C2">
-        <v>-1.442075288570562</v>
+        <v>0.9249758352155775</v>
       </c>
       <c r="D2">
-        <v>0.7323982788014326</v>
+        <v>0.9676548679233398</v>
       </c>
       <c r="E2">
-        <v>-1.968976894553211</v>
+        <v>0.9558943646929047</v>
       </c>
       <c r="F2">
-        <v>0.05009209661743455</v>
+        <v>0.3399190240163537</v>
       </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>Case FE + Clash: Extortion</t>
+          <t>Case FE: Civilian targeting</t>
         </is>
       </c>
       <c r="B3" t="inlineStr">
@@ -1202,16 +1339,40 @@
         </is>
       </c>
       <c r="C3">
-        <v>2.018509843327398</v>
+        <v>4.088173688318293</v>
       </c>
       <c r="D3">
-        <v>0.758960924512239</v>
+        <v>0.6918973308035009</v>
       </c>
       <c r="E3">
-        <v>2.65957018093472</v>
+        <v>5.908642086493807</v>
       </c>
       <c r="F3">
-        <v>0.008344407568899728</v>
+        <v>9.625368238438398E-09</v>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" t="inlineStr">
+        <is>
+          <t>Case FE: Civilian targeting</t>
+        </is>
+      </c>
+      <c r="B4" t="inlineStr">
+        <is>
+          <t>treatment_dummy:clash_dummy</t>
+        </is>
+      </c>
+      <c r="C4">
+        <v>-1.468538291674597</v>
+      </c>
+      <c r="D4">
+        <v>1.186519401300277</v>
+      </c>
+      <c r="E4">
+        <v>-1.237685865115448</v>
+      </c>
+      <c r="F4">
+        <v>0.2168302554862923</v>
       </c>
     </row>
   </sheetData>
@@ -1259,73 +1420,73 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>General OLS + Clash: Political violence</t>
+          <t>Case FE: Homicide</t>
         </is>
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>(Intercept)</t>
+          <t>treatment_dummy</t>
         </is>
       </c>
       <c r="C2">
-        <v>7.300437164798683</v>
+        <v>0.097456426219519</v>
       </c>
       <c r="D2">
-        <v>0.8102246295815889</v>
+        <v>1.437330746881344</v>
       </c>
       <c r="E2">
-        <v>9.010386623977018</v>
+        <v>0.06780375806401942</v>
       </c>
       <c r="F2">
-        <v>2.674477800475242E-17</v>
+        <v>0.9459924099961009</v>
       </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>General OLS + Clash: Political violence</t>
+          <t>Case FE: Homicide</t>
         </is>
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>treatment_dummy</t>
+          <t>clash_dummy</t>
         </is>
       </c>
       <c r="C3">
-        <v>-1.924051837861118</v>
+        <v>5.701920588910062</v>
       </c>
       <c r="D3">
-        <v>1.051582159888086</v>
+        <v>1.058826032372285</v>
       </c>
       <c r="E3">
-        <v>-1.829673335334906</v>
+        <v>5.385134492901529</v>
       </c>
       <c r="F3">
-        <v>0.06831135897813803</v>
+        <v>1.583566456239743E-07</v>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>General OLS + Clash: Political violence</t>
+          <t>Case FE: Homicide</t>
         </is>
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>clash_dummy</t>
+          <t>treatment_dummy:clash_dummy</t>
         </is>
       </c>
       <c r="C4">
-        <v>2.620862065819829</v>
+        <v>-2.316566990460848</v>
       </c>
       <c r="D4">
-        <v>0.9823936117597569</v>
+        <v>1.858507446772427</v>
       </c>
       <c r="E4">
-        <v>2.667832968829155</v>
+        <v>-1.246466348296807</v>
       </c>
       <c r="F4">
-        <v>0.008057624021933175</v>
+        <v>0.2136816164305728</v>
       </c>
     </row>
   </sheetData>
@@ -1373,73 +1534,73 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>General OLS + Clash: Civilian targeting</t>
+          <t>Case FE: Terrorism</t>
         </is>
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>(Intercept)</t>
+          <t>treatment_dummy</t>
         </is>
       </c>
       <c r="C2">
-        <v>3.359439737336234</v>
+        <v>-3.272925618639001</v>
       </c>
       <c r="D2">
-        <v>0.5244164426780868</v>
+        <v>1.970149059202227</v>
       </c>
       <c r="E2">
-        <v>6.406053403246219</v>
+        <v>-1.661257864399513</v>
       </c>
       <c r="F2">
-        <v>5.91194058926796E-10</v>
+        <v>0.0988836044867865</v>
       </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>General OLS + Clash: Civilian targeting</t>
+          <t>Case FE: Terrorism</t>
         </is>
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>treatment_dummy</t>
+          <t>clash_dummy</t>
         </is>
       </c>
       <c r="C3">
-        <v>-0.4672848266293707</v>
+        <v>-1.837952926941751</v>
       </c>
       <c r="D3">
-        <v>0.6806346725809042</v>
+        <v>0.9676912629951592</v>
       </c>
       <c r="E3">
-        <v>-0.6865427893314185</v>
+        <v>-1.899317475754605</v>
       </c>
       <c r="F3">
-        <v>0.49291200260067</v>
+        <v>0.05956518518057766</v>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>General OLS + Clash: Civilian targeting</t>
+          <t>Case FE: Terrorism</t>
         </is>
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>clash_dummy</t>
+          <t>treatment_dummy:clash_dummy</t>
         </is>
       </c>
       <c r="C4">
-        <v>2.801265723376451</v>
+        <v>2.579243021943121</v>
       </c>
       <c r="D4">
-        <v>0.6358525085256629</v>
+        <v>2.128727852504146</v>
       </c>
       <c r="E4">
-        <v>4.405527517492513</v>
+        <v>1.211635869239465</v>
       </c>
       <c r="F4">
-        <v>1.480005084391923E-05</v>
+        <v>0.2276784235571214</v>
       </c>
     </row>
   </sheetData>
@@ -1487,73 +1648,73 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>General OLS + Clash: Homicides</t>
+          <t>Case FE: Extortion</t>
         </is>
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>(Intercept)</t>
+          <t>treatment_dummy</t>
         </is>
       </c>
       <c r="C2">
-        <v>8.09213142694821</v>
+        <v>2.401639789790406</v>
       </c>
       <c r="D2">
-        <v>0.7415848461278788</v>
+        <v>1.161156681218406</v>
       </c>
       <c r="E2">
-        <v>10.91194280627574</v>
+        <v>2.068316729892436</v>
       </c>
       <c r="F2">
-        <v>3.210880042686441E-23</v>
+        <v>0.03967281101596914</v>
       </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>General OLS + Clash: Homicides</t>
+          <t>Case FE: Extortion</t>
         </is>
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>treatment_dummy</t>
+          <t>clash_dummy</t>
         </is>
       </c>
       <c r="C3">
-        <v>0.9107092131426942</v>
+        <v>3.82708779679586</v>
       </c>
       <c r="D3">
-        <v>1.018924668847289</v>
+        <v>0.8524974832643961</v>
       </c>
       <c r="E3">
-        <v>0.8937944491745216</v>
+        <v>4.48926580069318</v>
       </c>
       <c r="F3">
-        <v>0.3722249406019651</v>
+        <v>1.106292805431552E-05</v>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>General OLS + Clash: Homicides</t>
+          <t>Case FE: Extortion</t>
         </is>
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>clash_dummy</t>
+          <t>treatment_dummy:clash_dummy</t>
         </is>
       </c>
       <c r="C4">
-        <v>0.343318114638353</v>
+        <v>-6.237761858468893</v>
       </c>
       <c r="D4">
-        <v>0.9150595880409167</v>
+        <v>1.492593382725984</v>
       </c>
       <c r="E4">
-        <v>0.3751866207679161</v>
+        <v>-4.179143449689302</v>
       </c>
       <c r="F4">
-        <v>0.7078151487699633</v>
+        <v>4.089977077702876E-05</v>
       </c>
     </row>
   </sheetData>
@@ -1601,7 +1762,7 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>Pooled OLS + clash</t>
+          <t>OLS + clash</t>
         </is>
       </c>
       <c r="B2" t="inlineStr">
@@ -1625,7 +1786,7 @@
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>Pooled OLS + clash</t>
+          <t>OLS + clash</t>
         </is>
       </c>
       <c r="B3" t="inlineStr">
@@ -1649,7 +1810,7 @@
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>Pooled OLS + clash</t>
+          <t>OLS + clash</t>
         </is>
       </c>
       <c r="B4" t="inlineStr">
@@ -1715,73 +1876,73 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>General OLS + Clash: Terrorism</t>
+          <t>TWFE: Political violence</t>
         </is>
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>(Intercept)</t>
+          <t>treatment_dummy</t>
         </is>
       </c>
       <c r="C2">
-        <v>6.868629023820324</v>
+        <v>4.541174009773997</v>
       </c>
       <c r="D2">
-        <v>0.6253946141455978</v>
+        <v>1.859917737603292</v>
       </c>
       <c r="E2">
-        <v>10.9828720434443</v>
+        <v>2.441599387952393</v>
       </c>
       <c r="F2">
-        <v>9.161725945289539E-21</v>
+        <v>0.01552368019789591</v>
       </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>General OLS + Clash: Terrorism</t>
+          <t>TWFE: Political violence</t>
         </is>
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>treatment_dummy</t>
+          <t>clash_dummy</t>
         </is>
       </c>
       <c r="C3">
-        <v>-1.34006905451122</v>
+        <v>8.045044814057947</v>
       </c>
       <c r="D3">
-        <v>0.8903251969159173</v>
+        <v>1.187697975841139</v>
       </c>
       <c r="E3">
-        <v>-1.505145602026331</v>
+        <v>6.773645301837251</v>
       </c>
       <c r="F3">
-        <v>0.1344769589800681</v>
+        <v>1.47735849004418E-10</v>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>General OLS + Clash: Terrorism</t>
+          <t>TWFE: Political violence</t>
         </is>
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>clash_dummy</t>
+          <t>treatment_dummy:clash_dummy</t>
         </is>
       </c>
       <c r="C4">
-        <v>-2.54747672025948</v>
+        <v>-4.951871872995454</v>
       </c>
       <c r="D4">
-        <v>0.8342277167158826</v>
+        <v>1.835529871382409</v>
       </c>
       <c r="E4">
-        <v>-3.053694655804738</v>
+        <v>-2.697788769444546</v>
       </c>
       <c r="F4">
-        <v>0.002693308857944394</v>
+        <v>0.007598403917769804</v>
       </c>
     </row>
   </sheetData>
@@ -1829,73 +1990,73 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>General OLS + Clash: Extortion</t>
+          <t>TWFE: Civilian targeting</t>
         </is>
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>(Intercept)</t>
+          <t>treatment_dummy</t>
         </is>
       </c>
       <c r="C2">
-        <v>9.782597235910247</v>
+        <v>2.303481476187562</v>
       </c>
       <c r="D2">
-        <v>0.6469752497464141</v>
+        <v>1.274413913235212</v>
       </c>
       <c r="E2">
-        <v>15.12051232213998</v>
+        <v>1.807482994547644</v>
       </c>
       <c r="F2">
-        <v>6.233867340594593E-37</v>
+        <v>0.07224412430685603</v>
       </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>General OLS + Clash: Extortion</t>
+          <t>TWFE: Civilian targeting</t>
         </is>
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>treatment_dummy</t>
+          <t>clash_dummy</t>
         </is>
       </c>
       <c r="C3">
-        <v>0.9839449015608172</v>
+        <v>6.34653871917649</v>
       </c>
       <c r="D3">
-        <v>0.9035717200942001</v>
+        <v>0.8138095543320698</v>
       </c>
       <c r="E3">
-        <v>1.088950527865389</v>
+        <v>7.798555184554671</v>
       </c>
       <c r="F3">
-        <v>0.2772456769196435</v>
+        <v>3.81941965490486E-13</v>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>General OLS + Clash: Extortion</t>
+          <t>TWFE: Civilian targeting</t>
         </is>
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>clash_dummy</t>
+          <t>treatment_dummy:clash_dummy</t>
         </is>
       </c>
       <c r="C4">
-        <v>-2.843555423131863</v>
+        <v>-1.431227685670486</v>
       </c>
       <c r="D4">
-        <v>0.8333169338511409</v>
+        <v>1.257703369861362</v>
       </c>
       <c r="E4">
-        <v>-3.412333660364352</v>
+        <v>-1.13796919048428</v>
       </c>
       <c r="F4">
-        <v>0.0007533900203768379</v>
+        <v>0.2565440316948227</v>
       </c>
     </row>
   </sheetData>
@@ -1905,7 +2066,7 @@
 
 <file path=xl/worksheets/sheet22.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:F3"/>
+  <dimension ref="A1:F4"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <sheetData>
     <row r="1" s="1" customFormat="1">
@@ -1943,7 +2104,7 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>TWFE + Clash: Political violence</t>
+          <t>TWFE: Homicide</t>
         </is>
       </c>
       <c r="B2" t="inlineStr">
@@ -1952,22 +2113,22 @@
         </is>
       </c>
       <c r="C2">
-        <v>0.4574076593902843</v>
+        <v>2.116785029283085</v>
       </c>
       <c r="D2">
-        <v>1.098026078949257</v>
+        <v>2.175362005772684</v>
       </c>
       <c r="E2">
-        <v>0.4165726735998795</v>
+        <v>0.9730725385778752</v>
       </c>
       <c r="F2">
-        <v>0.6774515301263804</v>
+        <v>0.3318997833758752</v>
       </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>TWFE + Clash: Political violence</t>
+          <t>TWFE: Homicide</t>
         </is>
       </c>
       <c r="B3" t="inlineStr">
@@ -1976,16 +2137,40 @@
         </is>
       </c>
       <c r="C3">
-        <v>6.296994458504234</v>
+        <v>4.775679072701792</v>
       </c>
       <c r="D3">
-        <v>1.011356175619191</v>
+        <v>1.465241388054381</v>
       </c>
       <c r="E3">
-        <v>6.226287642579501</v>
+        <v>3.259312159509207</v>
       </c>
       <c r="F3">
-        <v>2.895348847642836E-09</v>
+        <v>0.001348958260422087</v>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" t="inlineStr">
+        <is>
+          <t>TWFE: Homicide</t>
+        </is>
+      </c>
+      <c r="B4" t="inlineStr">
+        <is>
+          <t>treatment_dummy:clash_dummy</t>
+        </is>
+      </c>
+      <c r="C4">
+        <v>-0.7230535374192826</v>
+      </c>
+      <c r="D4">
+        <v>2.195187946079009</v>
+      </c>
+      <c r="E4">
+        <v>-0.3293811533134477</v>
+      </c>
+      <c r="F4">
+        <v>0.7422730765445325</v>
       </c>
     </row>
   </sheetData>
@@ -1995,7 +2180,7 @@
 
 <file path=xl/worksheets/sheet23.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:F3"/>
+  <dimension ref="A1:F4"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <sheetData>
     <row r="1" s="1" customFormat="1">
@@ -2033,7 +2218,7 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>TWFE + Clash: Civilian targeting</t>
+          <t>TWFE: Terrorism</t>
         </is>
       </c>
       <c r="B2" t="inlineStr">
@@ -2042,22 +2227,22 @@
         </is>
       </c>
       <c r="C2">
-        <v>1.123160253751917</v>
+        <v>-2.907481680602449</v>
       </c>
       <c r="D2">
-        <v>0.7410431780027535</v>
+        <v>3.702005378171124</v>
       </c>
       <c r="E2">
-        <v>1.51564751837948</v>
+        <v>-0.7853801881937869</v>
       </c>
       <c r="F2">
-        <v>0.1312361651412578</v>
+        <v>0.436172065263742</v>
       </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>TWFE + Clash: Civilian targeting</t>
+          <t>TWFE: Terrorism</t>
         </is>
       </c>
       <c r="B3" t="inlineStr">
@@ -2066,16 +2251,40 @@
         </is>
       </c>
       <c r="C3">
-        <v>5.841303905154292</v>
+        <v>0.8621448273735073</v>
       </c>
       <c r="D3">
-        <v>0.6825508144494546</v>
+        <v>1.683959806824303</v>
       </c>
       <c r="E3">
-        <v>8.558049864559734</v>
+        <v>0.5119747062130797</v>
       </c>
       <c r="F3">
-        <v>3.468663819464876E-15</v>
+        <v>0.6110661112653426</v>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" t="inlineStr">
+        <is>
+          <t>TWFE: Terrorism</t>
+        </is>
+      </c>
+      <c r="B4" t="inlineStr">
+        <is>
+          <t>treatment_dummy:clash_dummy</t>
+        </is>
+      </c>
+      <c r="C4">
+        <v>0.9276074056769561</v>
+      </c>
+      <c r="D4">
+        <v>2.88123871640397</v>
+      </c>
+      <c r="E4">
+        <v>0.3219474319832439</v>
+      </c>
+      <c r="F4">
+        <v>0.7489201266852989</v>
       </c>
     </row>
   </sheetData>
@@ -2085,276 +2294,6 @@
 
 <file path=xl/worksheets/sheet24.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:F3"/>
-  <sheetFormatPr defaultRowHeight="15"/>
-  <sheetData>
-    <row r="1" s="1" customFormat="1">
-      <c r="A1" s="1" t="inlineStr">
-        <is>
-          <t>model</t>
-        </is>
-      </c>
-      <c r="B1" s="1" t="inlineStr">
-        <is>
-          <t>term</t>
-        </is>
-      </c>
-      <c r="C1" s="1" t="inlineStr">
-        <is>
-          <t>Estimate</t>
-        </is>
-      </c>
-      <c r="D1" s="1" t="inlineStr">
-        <is>
-          <t>Std. Error</t>
-        </is>
-      </c>
-      <c r="E1" s="1" t="inlineStr">
-        <is>
-          <t>t value</t>
-        </is>
-      </c>
-      <c r="F1" s="1" t="inlineStr">
-        <is>
-          <t>Pr(&gt;|t|)</t>
-        </is>
-      </c>
-    </row>
-    <row r="2">
-      <c r="A2" t="inlineStr">
-        <is>
-          <t>TWFE + Clash: Homicides</t>
-        </is>
-      </c>
-      <c r="B2" t="inlineStr">
-        <is>
-          <t>treatment_dummy</t>
-        </is>
-      </c>
-      <c r="C2">
-        <v>1.559255671921433</v>
-      </c>
-      <c r="D2">
-        <v>1.362856381766952</v>
-      </c>
-      <c r="E2">
-        <v>1.144108574301753</v>
-      </c>
-      <c r="F2">
-        <v>0.2541776184654491</v>
-      </c>
-    </row>
-    <row r="3">
-      <c r="A3" t="inlineStr">
-        <is>
-          <t>TWFE + Clash: Homicides</t>
-        </is>
-      </c>
-      <c r="B3" t="inlineStr">
-        <is>
-          <t>clash_dummy</t>
-        </is>
-      </c>
-      <c r="C3">
-        <v>4.486724484877757</v>
-      </c>
-      <c r="D3">
-        <v>1.170537284218909</v>
-      </c>
-      <c r="E3">
-        <v>3.833047050587301</v>
-      </c>
-      <c r="F3">
-        <v>0.0001776189018111053</v>
-      </c>
-    </row>
-  </sheetData>
-  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-</worksheet>
-</file>
-
-<file path=xl/worksheets/sheet25.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:F3"/>
-  <sheetFormatPr defaultRowHeight="15"/>
-  <sheetData>
-    <row r="1" s="1" customFormat="1">
-      <c r="A1" s="1" t="inlineStr">
-        <is>
-          <t>model</t>
-        </is>
-      </c>
-      <c r="B1" s="1" t="inlineStr">
-        <is>
-          <t>term</t>
-        </is>
-      </c>
-      <c r="C1" s="1" t="inlineStr">
-        <is>
-          <t>Estimate</t>
-        </is>
-      </c>
-      <c r="D1" s="1" t="inlineStr">
-        <is>
-          <t>Std. Error</t>
-        </is>
-      </c>
-      <c r="E1" s="1" t="inlineStr">
-        <is>
-          <t>t value</t>
-        </is>
-      </c>
-      <c r="F1" s="1" t="inlineStr">
-        <is>
-          <t>Pr(&gt;|t|)</t>
-        </is>
-      </c>
-    </row>
-    <row r="2">
-      <c r="A2" t="inlineStr">
-        <is>
-          <t>TWFE + Clash: Terrorism</t>
-        </is>
-      </c>
-      <c r="B2" t="inlineStr">
-        <is>
-          <t>treatment_dummy</t>
-        </is>
-      </c>
-      <c r="C2">
-        <v>-1.822566945606037</v>
-      </c>
-      <c r="D2">
-        <v>1.51825122944914</v>
-      </c>
-      <c r="E2">
-        <v>-1.200438313669149</v>
-      </c>
-      <c r="F2">
-        <v>0.2358601540580138</v>
-      </c>
-    </row>
-    <row r="3">
-      <c r="A3" t="inlineStr">
-        <is>
-          <t>TWFE + Clash: Terrorism</t>
-        </is>
-      </c>
-      <c r="B3" t="inlineStr">
-        <is>
-          <t>clash_dummy</t>
-        </is>
-      </c>
-      <c r="C3">
-        <v>1.210274619981761</v>
-      </c>
-      <c r="D3">
-        <v>1.27880320160346</v>
-      </c>
-      <c r="E3">
-        <v>0.9464119408398626</v>
-      </c>
-      <c r="F3">
-        <v>0.3486787470970519</v>
-      </c>
-    </row>
-  </sheetData>
-  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-</worksheet>
-</file>
-
-<file path=xl/worksheets/sheet26.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:F3"/>
-  <sheetFormatPr defaultRowHeight="15"/>
-  <sheetData>
-    <row r="1" s="1" customFormat="1">
-      <c r="A1" s="1" t="inlineStr">
-        <is>
-          <t>model</t>
-        </is>
-      </c>
-      <c r="B1" s="1" t="inlineStr">
-        <is>
-          <t>term</t>
-        </is>
-      </c>
-      <c r="C1" s="1" t="inlineStr">
-        <is>
-          <t>Estimate</t>
-        </is>
-      </c>
-      <c r="D1" s="1" t="inlineStr">
-        <is>
-          <t>Std. Error</t>
-        </is>
-      </c>
-      <c r="E1" s="1" t="inlineStr">
-        <is>
-          <t>t value</t>
-        </is>
-      </c>
-      <c r="F1" s="1" t="inlineStr">
-        <is>
-          <t>Pr(&gt;|t|)</t>
-        </is>
-      </c>
-    </row>
-    <row r="2">
-      <c r="A2" t="inlineStr">
-        <is>
-          <t>TWFE + Clash: Extortion</t>
-        </is>
-      </c>
-      <c r="B2" t="inlineStr">
-        <is>
-          <t>treatment_dummy</t>
-        </is>
-      </c>
-      <c r="C2">
-        <v>-0.3744928745834384</v>
-      </c>
-      <c r="D2">
-        <v>1.264968782462296</v>
-      </c>
-      <c r="E2">
-        <v>-0.2960491039585006</v>
-      </c>
-      <c r="F2">
-        <v>0.7676161539395028</v>
-      </c>
-    </row>
-    <row r="3">
-      <c r="A3" t="inlineStr">
-        <is>
-          <t>TWFE + Clash: Extortion</t>
-        </is>
-      </c>
-      <c r="B3" t="inlineStr">
-        <is>
-          <t>clash_dummy</t>
-        </is>
-      </c>
-      <c r="C3">
-        <v>1.753777102765306</v>
-      </c>
-      <c r="D3">
-        <v>1.06918234926669</v>
-      </c>
-      <c r="E3">
-        <v>1.640297470275443</v>
-      </c>
-      <c r="F3">
-        <v>0.1031109126189756</v>
-      </c>
-    </row>
-  </sheetData>
-  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-</worksheet>
-</file>
-
-<file path=xl/worksheets/sheet27.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
   <dimension ref="A1:F4"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <sheetData>
@@ -2393,7 +2332,7 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>TWFE + Clash + Interaction: Political violence</t>
+          <t>TWFE: Extortion</t>
         </is>
       </c>
       <c r="B2" t="inlineStr">
@@ -2402,22 +2341,22 @@
         </is>
       </c>
       <c r="C2">
-        <v>4.541174009773997</v>
+        <v>6.673331458059105</v>
       </c>
       <c r="D2">
-        <v>1.859917737603292</v>
+        <v>2.058062077006282</v>
       </c>
       <c r="E2">
-        <v>2.441599387952393</v>
+        <v>3.242531667347143</v>
       </c>
       <c r="F2">
-        <v>0.01552368019789591</v>
+        <v>0.001472330207037977</v>
       </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>TWFE + Clash + Interaction: Political violence</t>
+          <t>TWFE: Extortion</t>
         </is>
       </c>
       <c r="B3" t="inlineStr">
@@ -2426,22 +2365,22 @@
         </is>
       </c>
       <c r="C3">
-        <v>8.045044814057947</v>
+        <v>5.397012923803707</v>
       </c>
       <c r="D3">
-        <v>1.187697975841139</v>
+        <v>1.331675771531013</v>
       </c>
       <c r="E3">
-        <v>6.773645301837251</v>
+        <v>4.052798015239717</v>
       </c>
       <c r="F3">
-        <v>1.47735849004418E-10</v>
+        <v>8.247757316626191E-05</v>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>TWFE + Clash + Interaction: Political violence</t>
+          <t>TWFE: Extortion</t>
         </is>
       </c>
       <c r="B4" t="inlineStr">
@@ -2450,244 +2389,16 @@
         </is>
       </c>
       <c r="C4">
-        <v>-4.951871872995454</v>
+        <v>-8.241752064753952</v>
       </c>
       <c r="D4">
-        <v>1.835529871382409</v>
+        <v>1.957146359299602</v>
       </c>
       <c r="E4">
-        <v>-2.697788769444546</v>
+        <v>-4.211106658218142</v>
       </c>
       <c r="F4">
-        <v>0.007598403917769804</v>
-      </c>
-    </row>
-  </sheetData>
-  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-</worksheet>
-</file>
-
-<file path=xl/worksheets/sheet28.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:F4"/>
-  <sheetFormatPr defaultRowHeight="15"/>
-  <sheetData>
-    <row r="1" s="1" customFormat="1">
-      <c r="A1" s="1" t="inlineStr">
-        <is>
-          <t>model</t>
-        </is>
-      </c>
-      <c r="B1" s="1" t="inlineStr">
-        <is>
-          <t>term</t>
-        </is>
-      </c>
-      <c r="C1" s="1" t="inlineStr">
-        <is>
-          <t>Estimate</t>
-        </is>
-      </c>
-      <c r="D1" s="1" t="inlineStr">
-        <is>
-          <t>Std. Error</t>
-        </is>
-      </c>
-      <c r="E1" s="1" t="inlineStr">
-        <is>
-          <t>t value</t>
-        </is>
-      </c>
-      <c r="F1" s="1" t="inlineStr">
-        <is>
-          <t>Pr(&gt;|t|)</t>
-        </is>
-      </c>
-    </row>
-    <row r="2">
-      <c r="A2" t="inlineStr">
-        <is>
-          <t>TWFE + Clash + Interaction: Civilian targeting</t>
-        </is>
-      </c>
-      <c r="B2" t="inlineStr">
-        <is>
-          <t>treatment_dummy</t>
-        </is>
-      </c>
-      <c r="C2">
-        <v>2.303481476187562</v>
-      </c>
-      <c r="D2">
-        <v>1.274413913235212</v>
-      </c>
-      <c r="E2">
-        <v>1.807482994547644</v>
-      </c>
-      <c r="F2">
-        <v>0.07224412430685603</v>
-      </c>
-    </row>
-    <row r="3">
-      <c r="A3" t="inlineStr">
-        <is>
-          <t>TWFE + Clash + Interaction: Civilian targeting</t>
-        </is>
-      </c>
-      <c r="B3" t="inlineStr">
-        <is>
-          <t>clash_dummy</t>
-        </is>
-      </c>
-      <c r="C3">
-        <v>6.34653871917649</v>
-      </c>
-      <c r="D3">
-        <v>0.8138095543320698</v>
-      </c>
-      <c r="E3">
-        <v>7.798555184554671</v>
-      </c>
-      <c r="F3">
-        <v>3.81941965490486E-13</v>
-      </c>
-    </row>
-    <row r="4">
-      <c r="A4" t="inlineStr">
-        <is>
-          <t>TWFE + Clash + Interaction: Civilian targeting</t>
-        </is>
-      </c>
-      <c r="B4" t="inlineStr">
-        <is>
-          <t>treatment_dummy:clash_dummy</t>
-        </is>
-      </c>
-      <c r="C4">
-        <v>-1.431227685670486</v>
-      </c>
-      <c r="D4">
-        <v>1.257703369861362</v>
-      </c>
-      <c r="E4">
-        <v>-1.13796919048428</v>
-      </c>
-      <c r="F4">
-        <v>0.2565440316948227</v>
-      </c>
-    </row>
-  </sheetData>
-  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-</worksheet>
-</file>
-
-<file path=xl/worksheets/sheet29.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:F4"/>
-  <sheetFormatPr defaultRowHeight="15"/>
-  <sheetData>
-    <row r="1" s="1" customFormat="1">
-      <c r="A1" s="1" t="inlineStr">
-        <is>
-          <t>model</t>
-        </is>
-      </c>
-      <c r="B1" s="1" t="inlineStr">
-        <is>
-          <t>term</t>
-        </is>
-      </c>
-      <c r="C1" s="1" t="inlineStr">
-        <is>
-          <t>Estimate</t>
-        </is>
-      </c>
-      <c r="D1" s="1" t="inlineStr">
-        <is>
-          <t>Std. Error</t>
-        </is>
-      </c>
-      <c r="E1" s="1" t="inlineStr">
-        <is>
-          <t>t value</t>
-        </is>
-      </c>
-      <c r="F1" s="1" t="inlineStr">
-        <is>
-          <t>Pr(&gt;|t|)</t>
-        </is>
-      </c>
-    </row>
-    <row r="2">
-      <c r="A2" t="inlineStr">
-        <is>
-          <t>TWFE + Clash + Interaction: Homicides</t>
-        </is>
-      </c>
-      <c r="B2" t="inlineStr">
-        <is>
-          <t>treatment_dummy</t>
-        </is>
-      </c>
-      <c r="C2">
-        <v>2.116785029283085</v>
-      </c>
-      <c r="D2">
-        <v>2.175362005772684</v>
-      </c>
-      <c r="E2">
-        <v>0.9730725385778752</v>
-      </c>
-      <c r="F2">
-        <v>0.3318997833758752</v>
-      </c>
-    </row>
-    <row r="3">
-      <c r="A3" t="inlineStr">
-        <is>
-          <t>TWFE + Clash + Interaction: Homicides</t>
-        </is>
-      </c>
-      <c r="B3" t="inlineStr">
-        <is>
-          <t>clash_dummy</t>
-        </is>
-      </c>
-      <c r="C3">
-        <v>4.775679072701792</v>
-      </c>
-      <c r="D3">
-        <v>1.465241388054381</v>
-      </c>
-      <c r="E3">
-        <v>3.259312159509207</v>
-      </c>
-      <c r="F3">
-        <v>0.001348958260422087</v>
-      </c>
-    </row>
-    <row r="4">
-      <c r="A4" t="inlineStr">
-        <is>
-          <t>TWFE + Clash + Interaction: Homicides</t>
-        </is>
-      </c>
-      <c r="B4" t="inlineStr">
-        <is>
-          <t>treatment_dummy:clash_dummy</t>
-        </is>
-      </c>
-      <c r="C4">
-        <v>-0.7230535374192826</v>
-      </c>
-      <c r="D4">
-        <v>2.195187946079009</v>
-      </c>
-      <c r="E4">
-        <v>-0.3293811533134477</v>
-      </c>
-      <c r="F4">
-        <v>0.7422730765445325</v>
+        <v>4.45681403737058E-05</v>
       </c>
     </row>
   </sheetData>
@@ -2735,7 +2446,7 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>Pooled OLS + clash + interaction</t>
+          <t>OLS + clash + interaction</t>
         </is>
       </c>
       <c r="B2" t="inlineStr">
@@ -2759,7 +2470,7 @@
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>Pooled OLS + clash + interaction</t>
+          <t>OLS + clash + interaction</t>
         </is>
       </c>
       <c r="B3" t="inlineStr">
@@ -2783,7 +2494,7 @@
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>Pooled OLS + clash + interaction</t>
+          <t>OLS + clash + interaction</t>
         </is>
       </c>
       <c r="B4" t="inlineStr">
@@ -2807,7 +2518,7 @@
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>Pooled OLS + clash + interaction</t>
+          <t>OLS + clash + interaction</t>
         </is>
       </c>
       <c r="B5" t="inlineStr">
@@ -2826,234 +2537,6 @@
       </c>
       <c r="F5">
         <v>0.009593770268973671</v>
-      </c>
-    </row>
-  </sheetData>
-  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-</worksheet>
-</file>
-
-<file path=xl/worksheets/sheet30.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:F4"/>
-  <sheetFormatPr defaultRowHeight="15"/>
-  <sheetData>
-    <row r="1" s="1" customFormat="1">
-      <c r="A1" s="1" t="inlineStr">
-        <is>
-          <t>model</t>
-        </is>
-      </c>
-      <c r="B1" s="1" t="inlineStr">
-        <is>
-          <t>term</t>
-        </is>
-      </c>
-      <c r="C1" s="1" t="inlineStr">
-        <is>
-          <t>Estimate</t>
-        </is>
-      </c>
-      <c r="D1" s="1" t="inlineStr">
-        <is>
-          <t>Std. Error</t>
-        </is>
-      </c>
-      <c r="E1" s="1" t="inlineStr">
-        <is>
-          <t>t value</t>
-        </is>
-      </c>
-      <c r="F1" s="1" t="inlineStr">
-        <is>
-          <t>Pr(&gt;|t|)</t>
-        </is>
-      </c>
-    </row>
-    <row r="2">
-      <c r="A2" t="inlineStr">
-        <is>
-          <t>TWFE + Clash + Interaction: Terrorism</t>
-        </is>
-      </c>
-      <c r="B2" t="inlineStr">
-        <is>
-          <t>treatment_dummy</t>
-        </is>
-      </c>
-      <c r="C2">
-        <v>-2.907481680602449</v>
-      </c>
-      <c r="D2">
-        <v>3.702005378171124</v>
-      </c>
-      <c r="E2">
-        <v>-0.7853801881937869</v>
-      </c>
-      <c r="F2">
-        <v>0.436172065263742</v>
-      </c>
-    </row>
-    <row r="3">
-      <c r="A3" t="inlineStr">
-        <is>
-          <t>TWFE + Clash + Interaction: Terrorism</t>
-        </is>
-      </c>
-      <c r="B3" t="inlineStr">
-        <is>
-          <t>clash_dummy</t>
-        </is>
-      </c>
-      <c r="C3">
-        <v>0.8621448273735073</v>
-      </c>
-      <c r="D3">
-        <v>1.683959806824303</v>
-      </c>
-      <c r="E3">
-        <v>0.5119747062130797</v>
-      </c>
-      <c r="F3">
-        <v>0.6110661112653426</v>
-      </c>
-    </row>
-    <row r="4">
-      <c r="A4" t="inlineStr">
-        <is>
-          <t>TWFE + Clash + Interaction: Terrorism</t>
-        </is>
-      </c>
-      <c r="B4" t="inlineStr">
-        <is>
-          <t>treatment_dummy:clash_dummy</t>
-        </is>
-      </c>
-      <c r="C4">
-        <v>0.9276074056769561</v>
-      </c>
-      <c r="D4">
-        <v>2.88123871640397</v>
-      </c>
-      <c r="E4">
-        <v>0.3219474319832439</v>
-      </c>
-      <c r="F4">
-        <v>0.7489201266852989</v>
-      </c>
-    </row>
-  </sheetData>
-  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-</worksheet>
-</file>
-
-<file path=xl/worksheets/sheet31.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:F4"/>
-  <sheetFormatPr defaultRowHeight="15"/>
-  <sheetData>
-    <row r="1" s="1" customFormat="1">
-      <c r="A1" s="1" t="inlineStr">
-        <is>
-          <t>model</t>
-        </is>
-      </c>
-      <c r="B1" s="1" t="inlineStr">
-        <is>
-          <t>term</t>
-        </is>
-      </c>
-      <c r="C1" s="1" t="inlineStr">
-        <is>
-          <t>Estimate</t>
-        </is>
-      </c>
-      <c r="D1" s="1" t="inlineStr">
-        <is>
-          <t>Std. Error</t>
-        </is>
-      </c>
-      <c r="E1" s="1" t="inlineStr">
-        <is>
-          <t>t value</t>
-        </is>
-      </c>
-      <c r="F1" s="1" t="inlineStr">
-        <is>
-          <t>Pr(&gt;|t|)</t>
-        </is>
-      </c>
-    </row>
-    <row r="2">
-      <c r="A2" t="inlineStr">
-        <is>
-          <t>TWFE + Clash + Interaction: Extortion</t>
-        </is>
-      </c>
-      <c r="B2" t="inlineStr">
-        <is>
-          <t>treatment_dummy</t>
-        </is>
-      </c>
-      <c r="C2">
-        <v>6.673331458059105</v>
-      </c>
-      <c r="D2">
-        <v>2.058062077006282</v>
-      </c>
-      <c r="E2">
-        <v>3.242531667347143</v>
-      </c>
-      <c r="F2">
-        <v>0.001472330207037977</v>
-      </c>
-    </row>
-    <row r="3">
-      <c r="A3" t="inlineStr">
-        <is>
-          <t>TWFE + Clash + Interaction: Extortion</t>
-        </is>
-      </c>
-      <c r="B3" t="inlineStr">
-        <is>
-          <t>clash_dummy</t>
-        </is>
-      </c>
-      <c r="C3">
-        <v>5.397012923803707</v>
-      </c>
-      <c r="D3">
-        <v>1.331675771531013</v>
-      </c>
-      <c r="E3">
-        <v>4.052798015239717</v>
-      </c>
-      <c r="F3">
-        <v>8.247757316626191E-05</v>
-      </c>
-    </row>
-    <row r="4">
-      <c r="A4" t="inlineStr">
-        <is>
-          <t>TWFE + Clash + Interaction: Extortion</t>
-        </is>
-      </c>
-      <c r="B4" t="inlineStr">
-        <is>
-          <t>treatment_dummy:clash_dummy</t>
-        </is>
-      </c>
-      <c r="C4">
-        <v>-8.241752064753952</v>
-      </c>
-      <c r="D4">
-        <v>1.957146359299602</v>
-      </c>
-      <c r="E4">
-        <v>-4.211106658218142</v>
-      </c>
-      <c r="F4">
-        <v>4.45681403737058E-05</v>
       </c>
     </row>
   </sheetData>
@@ -3437,7 +2920,7 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>TWFE + Clashes</t>
+          <t>TWFE + clash</t>
         </is>
       </c>
       <c r="B2" t="inlineStr">
@@ -3461,7 +2944,7 @@
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>TWFE + Clashes</t>
+          <t>TWFE + clash</t>
         </is>
       </c>
       <c r="B3" t="inlineStr">
@@ -3527,7 +3010,7 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>TWFE + Clashes + Interaction</t>
+          <t>TWFE + clash + interaction</t>
         </is>
       </c>
       <c r="B2" t="inlineStr">
@@ -3551,7 +3034,7 @@
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>TWFE + Clashes + Interaction</t>
+          <t>TWFE + clash + interaction</t>
         </is>
       </c>
       <c r="B3" t="inlineStr">
@@ -3575,7 +3058,7 @@
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>TWFE + Clashes + Interaction</t>
+          <t>TWFE + clash + interaction</t>
         </is>
       </c>
       <c r="B4" t="inlineStr">

</xml_diff>